<commit_message>
Organized and cleaned up some files
</commit_message>
<xml_diff>
--- a/correlation_graph.xlsx
+++ b/correlation_graph.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhuan08/Documents/Programming_Projects/oled-project-main/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhuan08/Programming Projects/oled-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9798C780-35A5-4D45-AE07-E428C29B0013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B07289AB-F639-AF4D-9800-4EAAC1B859D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1080" yWindow="1240" windowWidth="27640" windowHeight="16260" xr2:uid="{DF7F3765-FD89-0D40-8244-227DDC256222}"/>
   </bookViews>
@@ -278,7 +278,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{169D70F5-9DCE-074D-B85C-582E6FA1B98D}" type="CELLRANGE">
+                    <a:fld id="{994F712D-ECA3-5945-AEA7-489FCCC6B137}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -317,7 +317,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{D605D3AB-73A2-5940-A650-7492A6E4875A}" type="CELLRANGE">
+                    <a:fld id="{16304B7B-CD73-9144-A8FB-C3D0D4276162}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -356,7 +356,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{1F928A02-ECB1-A84F-A8F9-83F3C8E3830E}" type="CELLRANGE">
+                    <a:fld id="{612D8BD1-74DA-FF4A-B191-52E6597E6118}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -395,7 +395,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{3E41C0F0-F96C-5F45-8765-98DE6BE38356}" type="CELLRANGE">
+                    <a:fld id="{A904177C-BFAF-9E46-B5BA-2677712EE882}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -434,7 +434,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A18ADC4D-C668-7241-9CE3-C8F6DD4D38F2}" type="CELLRANGE">
+                    <a:fld id="{2358FBD4-921A-F747-A9A7-5F5AC4233164}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -473,7 +473,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{E8762B64-969F-4847-B983-6EAF9C2B4700}" type="CELLRANGE">
+                    <a:fld id="{BDC6C507-DCC4-9D4D-9D34-FCA0AC5D4255}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -512,7 +512,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{F7C3181B-2E1D-2240-A7C6-62AF9198387B}" type="CELLRANGE">
+                    <a:fld id="{14DB27D6-8B6E-8247-BB40-BEE197AC6B0A}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -551,7 +551,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{C56E235B-4BE6-F945-A73E-64FA06F33CAB}" type="CELLRANGE">
+                    <a:fld id="{A2496300-10FA-DD44-95D1-606EA20B406E}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -1654,16 +1654,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>220980</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>71120</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>7620</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>193040</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>279400</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>172720</xdr:rowOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>452120</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>91440</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>

<commit_message>
Updated Excel files, singlet_triplet_gap uses SMILES, optimization uses MOL2
</commit_message>
<xml_diff>
--- a/correlation_graph.xlsx
+++ b/correlation_graph.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhuan08/Programming Projects/oled-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B07289AB-F639-AF4D-9800-4EAAC1B859D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EC3A055-315D-0143-92E7-11A5D6F5A28C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1240" windowWidth="27640" windowHeight="16260" xr2:uid="{DF7F3765-FD89-0D40-8244-227DDC256222}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17000" xr2:uid="{DF7F3765-FD89-0D40-8244-227DDC256222}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>predicted</t>
   </si>
@@ -45,9 +45,6 @@
   </si>
   <si>
     <t>smiles</t>
-  </si>
-  <si>
-    <t>absorption_energy</t>
   </si>
   <si>
     <t>emission_energy</t>
@@ -278,7 +275,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{994F712D-ECA3-5945-AEA7-489FCCC6B137}" type="CELLRANGE">
+                    <a:fld id="{5B9DEAA0-A5E8-5B49-ACE8-D4760ACE85E7}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -317,7 +314,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{16304B7B-CD73-9144-A8FB-C3D0D4276162}" type="CELLRANGE">
+                    <a:fld id="{98628232-B2E2-4049-8A9C-F83DABF06D53}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -356,7 +353,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{612D8BD1-74DA-FF4A-B191-52E6597E6118}" type="CELLRANGE">
+                    <a:fld id="{027E1E81-108E-4748-84C7-D7A130E65344}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -395,7 +392,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A904177C-BFAF-9E46-B5BA-2677712EE882}" type="CELLRANGE">
+                    <a:fld id="{0122BDCE-EB46-E34E-8077-4C15A43B4F3E}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -434,7 +431,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{2358FBD4-921A-F747-A9A7-5F5AC4233164}" type="CELLRANGE">
+                    <a:fld id="{FE845039-0FDE-004E-972C-5B19D5B7189D}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -473,7 +470,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{BDC6C507-DCC4-9D4D-9D34-FCA0AC5D4255}" type="CELLRANGE">
+                    <a:fld id="{76BFEC26-94D7-7A47-8F6D-2FF9F045A6FB}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -512,7 +509,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{14DB27D6-8B6E-8247-BB40-BEE197AC6B0A}" type="CELLRANGE">
+                    <a:fld id="{F09E4D15-71ED-6640-8FC6-ABA5CE293BD5}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -551,7 +548,7 @@
                   <a:bodyPr/>
                   <a:lstStyle/>
                   <a:p>
-                    <a:fld id="{A2496300-10FA-DD44-95D1-606EA20B406E}" type="CELLRANGE">
+                    <a:fld id="{87B2E46D-C75E-2B40-B372-AB8282779BC1}" type="CELLRANGE">
                       <a:rPr lang="en-US"/>
                       <a:pPr/>
                       <a:t>[CELLRANGE]</a:t>
@@ -687,7 +684,7 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$D$2:$D$9</c:f>
+              <c:f>Sheet1!$C$2:$C$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
@@ -720,7 +717,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$E$2:$E$9</c:f>
+              <c:f>Sheet1!$D$2:$D$9</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
@@ -1654,16 +1651,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>7620</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>193040</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>78740</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>452120</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>91440</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>833120</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>162560</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2008,17 +2005,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{437ED259-CF5A-CE41-806D-66384DA86059}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -2029,145 +2026,118 @@
         <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>0</v>
+      <c r="B2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2.9520047246000001</v>
+      </c>
+      <c r="D2">
+        <v>2.6503877528168598</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="1" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="1">
-        <v>4.6090780086691501</v>
-      </c>
-      <c r="D2" s="1">
-        <v>2.9520047246000001</v>
-      </c>
-      <c r="E2">
-        <v>2.6503877528168598</v>
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1">
+        <v>3.0313984946992698</v>
+      </c>
+      <c r="D3">
+        <v>2.6649325265323101</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="1" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1">
-        <v>4.7870346885405501</v>
-      </c>
-      <c r="D3" s="1">
-        <v>3.0313984946992698</v>
-      </c>
-      <c r="E3">
-        <v>2.6649325265323101</v>
+      <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2.94499283689311</v>
+      </c>
+      <c r="D4">
+        <v>2.5977483063393199</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="1" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="1">
-        <v>4.6610600914736899</v>
-      </c>
-      <c r="D4" s="1">
+      <c r="B5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1">
+        <v>2.8968270661962601</v>
+      </c>
+      <c r="D5">
+        <v>2.54076374062651</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="1">
         <v>2.94499283689311</v>
       </c>
-      <c r="E4">
-        <v>2.5977483063393199</v>
+      <c r="D6">
+        <v>2.5876237612164901</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="1">
-        <v>4.6262760609402998</v>
-      </c>
-      <c r="D5" s="1">
-        <v>2.8968270661962601</v>
-      </c>
-      <c r="E5">
-        <v>2.54076374062651</v>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="1">
+        <v>2.58839662699791</v>
+      </c>
+      <c r="D7">
+        <v>1.83320161865776</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="1">
-        <v>4.7142280773079897</v>
-      </c>
-      <c r="D6" s="1">
-        <v>2.94499283689311</v>
-      </c>
-      <c r="E6">
-        <v>2.5876237612164901</v>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="1">
+        <v>3.6681715512781099</v>
+      </c>
+      <c r="D8">
+        <v>3.09235839203461</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="1">
-        <v>5.2535677300000003</v>
-      </c>
-      <c r="D7" s="1">
-        <v>2.58839662699791</v>
-      </c>
-      <c r="E7">
-        <v>1.83320161865776</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="1" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="1">
-        <v>5.1022303881975404</v>
-      </c>
-      <c r="D8" s="1">
-        <v>3.6681715512781099</v>
-      </c>
-      <c r="E8">
-        <v>3.09235839203461</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
+      <c r="B9" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>20</v>
-      </c>
       <c r="C9" s="1">
-        <v>4.6090780086691501</v>
-      </c>
-      <c r="D9" s="1">
         <v>2.5830041340249998</v>
       </c>
-      <c r="E9">
+      <c r="D9">
         <v>2.4915844109666501</v>
       </c>
     </row>

</xml_diff>